<commit_message>
TA report resend prepare
</commit_message>
<xml_diff>
--- a/2026_10/2026_10_02/LSLS/Navigation_SlackRecord.xlsx
+++ b/2026_10/2026_10_02/LSLS/Navigation_SlackRecord.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenalee\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenalee\work\2026_09\2026_10\2026_10_02\LSLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E07F2FE4-6261-49DD-A9EF-52C0F04E104A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E70FE1E7-C13D-49DA-AD61-7F300C3C458C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="27180" windowHeight="11205" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="27180" windowHeight="11205" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="reduction of salt.sugar" sheetId="1" r:id="rId1"/>
@@ -743,7 +743,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -781,13 +781,6 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -950,29 +943,29 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>

</xml_diff>